<commit_message>
Data Visualization with Seaborn
</commit_message>
<xml_diff>
--- a/2-Section- Basic Excel/data/04 Restaurant Sales.xlsx
+++ b/2-Section- Basic Excel/data/04 Restaurant Sales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8a6ce4a7617f1ad9/Desktop/courses/Data Analytics/2-Section- Basic Excel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{FB2AD424-2D60-4E2A-89EA-9C030A16242E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77B5EC31-BE83-4599-8B33-A3F0485335D3}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{FB2AD424-2D60-4E2A-89EA-9C030A16242E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AC8560E-E134-4D52-8865-95A038C0AA07}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{66301FCA-EA2A-4B3B-9A5C-535C597A10AA}"/>
   </bookViews>
@@ -40,8 +40,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5011" uniqueCount="1053">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5014" uniqueCount="1056">
   <si>
     <t>Transaction ID</t>
   </si>
@@ -3200,17 +3222,27 @@
   </si>
   <si>
     <t xml:space="preserve">Average rating </t>
+  </si>
+  <si>
+    <t>Count Delivery  Order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orders Types </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categories Orders </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="170" formatCode="[$$-C09]#,##0.00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3226,8 +3258,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3237,6 +3277,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF4472C4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3253,13 +3299,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3275,6 +3325,1886 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>Orders</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-IN" baseline="0"/>
+              <a:t> Types</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-IN"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-6654-4566-B043-F3904C32B282}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-6654-4566-B043-F3904C32B282}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-5C98-4E4F-BA3C-83A22D0BBA43}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="bg1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$F$2:$F$4</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Delivery</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Takeaway</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Dine-In</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$G$2:$G$4</c:f>
+              <c:numCache>
+                <c:formatCode>[$$-C09]#,##0.00</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>8457.3399999999529</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6594.4699999999757</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10747.639999999916</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5C98-4E4F-BA3C-83A22D0BBA43}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst>
+      <a:glow rad="63500">
+        <a:schemeClr val="accent4">
+          <a:satMod val="175000"/>
+          <a:alpha val="40000"/>
+        </a:schemeClr>
+      </a:glow>
+      <a:outerShdw blurRad="50800" dist="38100" dir="8100000" algn="tr" rotWithShape="0">
+        <a:prstClr val="black">
+          <a:alpha val="40000"/>
+        </a:prstClr>
+      </a:outerShdw>
+    </a:effectLst>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>Categories</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-IN" baseline="0"/>
+              <a:t> Orders </a:t>
+            </a:r>
+            <a:endParaRPr lang="en-IN"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.29578499562554683"/>
+          <c:y val="0.17171296296296298"/>
+          <c:w val="0.40287467191601051"/>
+          <c:h val="0.6714577865266842"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="bg1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$F$7:$F$10</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Main</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Beverage</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Appetizer</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Dessert</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$G$7:$G$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>11994.689999999902</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2382.4099999999985</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3872.629999999991</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2418.5699999999988</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F85B-4B02-8ACF-8D3913CDAF17}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="0"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst>
+      <a:glow rad="63500">
+        <a:schemeClr val="accent1">
+          <a:satMod val="175000"/>
+          <a:alpha val="40000"/>
+        </a:schemeClr>
+      </a:glow>
+      <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+        <a:prstClr val="black">
+          <a:alpha val="40000"/>
+        </a:prstClr>
+      </a:outerShdw>
+    </a:effectLst>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>604520</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>42333</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2D413B81-D065-D335-C20C-F9F710780A8B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>198120</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>90169</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>503767</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>5502</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{869212C1-CA0E-2611-495F-F5DCEEF03928}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -35648,13 +37578,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ECC67DF-3AE9-4D47-BE64-220802D2550B}">
-  <dimension ref="A2:B2"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.21875" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+      <c r="F1" s="4" t="s">
+        <v>1054</v>
+      </c>
+      <c r="G1" s="4"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1052</v>
       </c>
@@ -35662,8 +37600,89 @@
         <f>AVERAGE('Restaurant Sales'!J:J)</f>
         <v>3.9180000000000001</v>
       </c>
+      <c r="F2" t="str" cm="1">
+        <f t="array" ref="F2:F4">_xlfn.UNIQUE('Restaurant Sales'!D2:D1001)</f>
+        <v>Delivery</v>
+      </c>
+      <c r="G2" s="5">
+        <f>SUMIF('Restaurant Sales'!D:D, F2,'Restaurant Sales'!I:I)</f>
+        <v>8457.3399999999529</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B3">
+        <f>COUNTIF('Restaurant Sales'!D:D, "Delivery")</f>
+        <v>322</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Takeaway</v>
+      </c>
+      <c r="G3" s="5">
+        <f>SUMIF('Restaurant Sales'!D:D, F3,'Restaurant Sales'!I:I)</f>
+        <v>6594.4699999999757</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F4" t="str">
+        <v>Dine-In</v>
+      </c>
+      <c r="G4" s="5">
+        <f>SUMIF('Restaurant Sales'!D:D, F4,'Restaurant Sales'!I:I)</f>
+        <v>10747.639999999916</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+      <c r="F6" s="4" t="s">
+        <v>1055</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F7" t="str" cm="1">
+        <f t="array" ref="F7:F10">_xlfn.UNIQUE('Restaurant Sales'!F2:F1001)</f>
+        <v>Main</v>
+      </c>
+      <c r="G7">
+        <f ca="1">SUMIF('Restaurant Sales'!F1:F1001,F7,'Restaurant Sales'!I2:I1001)</f>
+        <v>11994.689999999902</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F8" t="str">
+        <v>Beverage</v>
+      </c>
+      <c r="G8">
+        <f>SUMIF('Restaurant Sales'!F2:F1002,F8,'Restaurant Sales'!I2:I1002)</f>
+        <v>2382.4099999999985</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F9" t="str">
+        <v>Appetizer</v>
+      </c>
+      <c r="G9">
+        <f>SUMIF('Restaurant Sales'!F3:F1003,F9,'Restaurant Sales'!I3:I1003)</f>
+        <v>3872.629999999991</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F10" t="str">
+        <v>Dessert</v>
+      </c>
+      <c r="G10">
+        <f>SUMIF('Restaurant Sales'!F4:F1004,F10,'Restaurant Sales'!I4:I1004)</f>
+        <v>2418.5699999999988</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F6:G6"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>